<commit_message>
. último commit sexta 03/11/2023
Código relaiza a captura e conversão de processos SIDA, previdênciário e outros para excel. Todavia, falta adicionar nas planilhas uma coluna com o número do processo.
</commit_message>
<xml_diff>
--- a/Saj_Ademir_codigo/processos.xlsx
+++ b/Saj_Ademir_codigo/processos.xlsx
@@ -14,56 +14,26 @@
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$A$3</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>5012989-45.2019.4.03.6182</t>
+    <t>5018620-67.2019.4.03.6182</t>
   </si>
   <si>
     <t>0503522-13.1995.4.03.6182</t>
   </si>
   <si>
-    <t>5018620-67.2019.4.03.6182</t>
+    <t>5012989-45.2019.4.03.6182</t>
   </si>
   <si>
-    <t>0057734-06.2016.4.03.6182</t>
-  </si>
-  <si>
-    <t>0001863-06.2007.4.03.6182</t>
-  </si>
-  <si>
-    <t>0033818-26.2005.4.03.6182</t>
-  </si>
-  <si>
-    <t>0028400-92.2014.4.03.6182</t>
-  </si>
-  <si>
-    <t>0016103-48.2017.4.03.6182</t>
-  </si>
-  <si>
-    <t>0517523-03.1995.4.03.6182</t>
-  </si>
-  <si>
-    <t>0020970-89.2014.4.03.6182</t>
-  </si>
-  <si>
-    <t>0055449-89.2006.4.03.6182</t>
-  </si>
-  <si>
-    <t>0502025-66.1992.4.03.6182</t>
-  </si>
-  <si>
-    <t>0013153-66.2017.4.03.6182</t>
-  </si>
-  <si>
-    <t>0059694-90.1999.4.03.6182</t>
-  </si>
-  <si>
-    <t>0034064-70.2015.4.03.6182</t>
+    <t>5002151-55.2020.4.03.6102</t>
   </si>
 </sst>
 </file>
@@ -101,7 +71,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -408,25 +378,26 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="49.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
+      <c r="A3" s="2" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -434,76 +405,16 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-    </row>
-    <row r="17" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-    </row>
-    <row r="18" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-    </row>
-    <row r="19" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-    </row>
+    <row r="5" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>